<commit_message>
update improvement in boxplot for monaco
</commit_message>
<xml_diff>
--- a/runs_eval/signal_controller_benchmark/full_performance_comparison.xlsx
+++ b/runs_eval/signal_controller_benchmark/full_performance_comparison.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Travid\updated_worst_case_MARL\runs_eval\signal_controller_benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80041CD9-47A4-41C2-BA9A-54A5C28B4487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B9E2C5-52DD-4A0E-B6C2-DF218A80B339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1448,76 +1448,100 @@
         <v>12</v>
       </c>
       <c r="B15" s="1">
-        <v>114.98</v>
+        <f>AVERAGE(B3:B14)</f>
+        <v>114.47749999999998</v>
       </c>
       <c r="C15" s="1">
-        <v>109.03</v>
+        <f>AVERAGE(C3:C14)</f>
+        <v>109.53333333333335</v>
       </c>
       <c r="D15" s="1">
-        <v>-4.32</v>
+        <f>(C15-B15)/B15*100</f>
+        <v>-4.3188981823210968</v>
       </c>
       <c r="E15" s="1">
-        <v>3.53</v>
+        <f t="shared" ref="D15:Y15" si="0">AVERAGE(E3:E14)</f>
+        <v>3.61</v>
       </c>
       <c r="F15" s="1">
-        <v>3.68</v>
+        <f t="shared" si="0"/>
+        <v>3.7691666666666666</v>
       </c>
       <c r="G15" s="1">
-        <v>4.38</v>
+        <f>(F15-E15)/E15*100</f>
+        <v>4.409048938134811</v>
       </c>
       <c r="H15" s="1">
-        <v>112.9</v>
+        <f t="shared" si="0"/>
+        <v>112.23166666666667</v>
       </c>
       <c r="I15" s="1">
-        <v>94.94</v>
+        <f t="shared" si="0"/>
+        <v>94.106666666666669</v>
       </c>
       <c r="J15" s="1">
-        <v>-16.149999999999999</v>
+        <f>(I15-H15)/H15*100</f>
+        <v>-16.1496309716509</v>
       </c>
       <c r="K15" s="1">
-        <v>3.52</v>
+        <f t="shared" si="0"/>
+        <v>3.6850000000000001</v>
       </c>
       <c r="L15" s="1">
-        <v>4.1500000000000004</v>
+        <f t="shared" si="0"/>
+        <v>4.1433333333333335</v>
       </c>
       <c r="M15" s="1">
-        <v>12.42</v>
+        <f>(L15-K15)/K15*100</f>
+        <v>12.437810945273636</v>
       </c>
       <c r="N15" s="1">
-        <v>159.63999999999999</v>
+        <f t="shared" si="0"/>
+        <v>159.47333333333336</v>
       </c>
       <c r="O15" s="1">
-        <v>104.15</v>
+        <f t="shared" si="0"/>
+        <v>104.73083333333335</v>
       </c>
       <c r="P15" s="1">
-        <v>-34.33</v>
+        <f>(O15-N15)/N15*100</f>
+        <v>-34.3270557250951</v>
       </c>
       <c r="Q15" s="1">
-        <v>3.63</v>
+        <f t="shared" si="0"/>
+        <v>3.6275000000000008</v>
       </c>
       <c r="R15" s="1">
-        <v>5.21</v>
+        <f t="shared" si="0"/>
+        <v>5.3791666666666664</v>
       </c>
       <c r="S15" s="1">
-        <v>48.22</v>
+        <f>(R15-Q15)/Q15*100</f>
+        <v>48.288536641396696</v>
       </c>
       <c r="T15" s="1">
-        <v>94.51</v>
+        <f t="shared" si="0"/>
+        <v>94.516666666666652</v>
       </c>
       <c r="U15" s="1">
-        <v>16.71</v>
+        <f t="shared" si="0"/>
+        <v>15.630833333333335</v>
       </c>
       <c r="V15" s="1">
-        <v>-83.46</v>
+        <f>(U15-T15)/T15*100</f>
+        <v>-83.462352318815022</v>
       </c>
       <c r="W15" s="1">
-        <v>3.86</v>
+        <f t="shared" si="0"/>
+        <v>4.0608333333333331</v>
       </c>
       <c r="X15" s="1">
-        <v>8.65</v>
+        <f t="shared" si="0"/>
+        <v>8.4816666666666674</v>
       </c>
       <c r="Y15" s="1">
-        <v>108.91</v>
+        <f>(X15-W15)/W15*100</f>
+        <v>108.86517545659761</v>
       </c>
     </row>
   </sheetData>

</xml_diff>